<commit_message>
Evaluating r for currency and index with perpetual = spot
</commit_message>
<xml_diff>
--- a/data_2026-08-13/df_dividends_announced.xlsx
+++ b/data_2026-08-13/df_dividends_announced.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,26 +608,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Т-Технологии, акция обыкновенная</t>
+          <t>ММЦБ, акция обыкновенная</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Московская Биржа, СПБ Биржа</t>
+          <t>Московская Биржа</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>T, TCSG</t>
+          <t>GEMA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Холдинги</t>
+          <t>Производство лекарств и биотехнологии</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4.7</v>
+        <v>2.74</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -635,24 +635,77 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>5.36</v>
+        <v>10.58</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46304</v>
+        <v>46290</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>46307</v>
+        <v>46293</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>46307</v>
+        <v>46293</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>46343</v>
+        <v>46328</v>
       </c>
       <c r="L4" t="n">
         <v>2026</v>
       </c>
       <c r="M4" t="inlineStr">
+        <is>
+          <t>6 месяцев (I полугодие)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Т-Технологии, акция обыкновенная</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Московская Биржа, СПБ Биржа</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>T, TCSG</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Холдинги</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>46343</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>6 месяцев (I полугодие)</t>
         </is>

</xml_diff>